<commit_message>
Big ahh Update for jet
</commit_message>
<xml_diff>
--- a/MAIN/Input Excel Sheets/Design Configurations/ASEN4138_Config_Jet.xlsx
+++ b/MAIN/Input Excel Sheets/Design Configurations/ASEN4138_Config_Jet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\GitHub\ASEN_Aircraft_Design\MAIN\Input Excel Sheets\Design Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85978DB0-2775-462B-8CCE-E2F5ECB74B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E78BBA41-0BCA-473F-ADB2-D86BCB2C56E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variable Reference" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <definedName name="MATERIALS" localSheetId="0">#REF!</definedName>
     <definedName name="MATERIALS">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -270,7 +270,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="250">
   <si>
     <t>Worksheet</t>
   </si>
@@ -1014,6 +1014,12 @@
   </si>
   <si>
     <t>JetSubmersible_conv1.5</t>
+  </si>
+  <si>
+    <t>Initial design configs</t>
+  </si>
+  <si>
+    <t>JetSubmersible_can1</t>
   </si>
 </sst>
 </file>
@@ -3778,7 +3784,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AMK15"/>
+  <dimension ref="A1:AMK19"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="21.21875" style="7" customWidth="1"/>
@@ -3966,11 +3972,11 @@
         <v>5.5</v>
       </c>
       <c r="H2" s="7">
-        <f>F2/G2</f>
+        <f t="shared" ref="H2:H11" si="0">F2/G2</f>
         <v>7.2727272727272725</v>
       </c>
       <c r="I2" s="7">
-        <f>((G2/2)^2)*3.1415+2.5</f>
+        <f t="shared" ref="I2:I11" si="1">((G2/2)^2)*3.1415+2.5</f>
         <v>26.257593750000002</v>
       </c>
       <c r="J2" s="7">
@@ -3987,24 +3993,24 @@
         <v>1</v>
       </c>
       <c r="N2" s="7">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="O2" s="7">
-        <f>N2*2</f>
-        <v>760</v>
+        <f t="shared" ref="O2:O11" si="2">N2*2</f>
+        <v>720</v>
       </c>
       <c r="P2" s="7">
-        <v>3.63</v>
+        <v>2</v>
       </c>
       <c r="Q2" s="7">
         <v>0.2</v>
       </c>
       <c r="R2" s="7">
-        <v>34</v>
+        <v>48.2</v>
       </c>
       <c r="S2" s="7">
-        <f>ATAN(TAN(R2*3.1415/180)-(1-Q2)/(2*(1+Q2)*P2))*180/3.1415</f>
-        <v>30.228351387955257</v>
+        <f>ATAN(TAN(R2*3.1415/180)-(1-Q2)/((1+Q2)*P2))*180/3.1415</f>
+        <v>38.134809329022481</v>
       </c>
       <c r="T2" s="7">
         <v>1.1000000000000001</v>
@@ -4013,7 +4019,7 @@
         <v>25</v>
       </c>
       <c r="V2" s="7">
-        <f>U2*2</f>
+        <f t="shared" ref="V2:V11" si="3">U2*2</f>
         <v>50</v>
       </c>
       <c r="W2" s="7">
@@ -4026,7 +4032,7 @@
         <v>32</v>
       </c>
       <c r="Z2" s="7">
-        <f>(2/3)*((2*U2)/((SQRT(W2*U2))*(1+X2)))*(1+X2+X2^2)/(1+X2)</f>
+        <f t="shared" ref="Z2:Z11" si="4">(2/3)*((2*U2)/((SQRT(W2*U2))*(1+X2)))*(1+X2+X2^2)/(1+X2)</f>
         <v>3.171014677825942</v>
       </c>
       <c r="AA2" s="7">
@@ -4057,7 +4063,7 @@
         <v>55</v>
       </c>
       <c r="AJ2" s="7">
-        <f>2*AI2</f>
+        <f t="shared" ref="AJ2:AJ11" si="5">2*AI2</f>
         <v>110</v>
       </c>
       <c r="AK2" s="7">
@@ -4070,7 +4076,7 @@
         <v>20</v>
       </c>
       <c r="AN2" s="7">
-        <f>(2/3)*((2*AI2)/((SQRT(AK2*AI2))*(1+AL2)))*(1+AL2+AL2^2)/(1+AL2)</f>
+        <f t="shared" ref="AN2:AN11" si="6">(2/3)*((2*AI2)/((SQRT(AK2*AI2))*(1+AL2)))*(1+AL2+AL2^2)/(1+AL2)</f>
         <v>6.9026671531786787</v>
       </c>
       <c r="AO2" s="7">
@@ -4121,11 +4127,11 @@
         <v>5.5</v>
       </c>
       <c r="H3" s="7">
-        <f>F3/G3</f>
+        <f t="shared" si="0"/>
         <v>7.2727272727272725</v>
       </c>
       <c r="I3" s="7">
-        <f>((G3/2)^2)*3.1415+2.5</f>
+        <f t="shared" si="1"/>
         <v>26.257593750000002</v>
       </c>
       <c r="J3" s="7">
@@ -4142,14 +4148,14 @@
         <v>1</v>
       </c>
       <c r="N3" s="7">
-        <v>360</v>
+        <v>450</v>
       </c>
       <c r="O3" s="7">
-        <f>N3*2</f>
-        <v>720</v>
+        <f t="shared" si="2"/>
+        <v>900</v>
       </c>
       <c r="P3" s="7">
-        <v>2.2000000000000002</v>
+        <v>1</v>
       </c>
       <c r="Q3" s="7">
         <v>0.2</v>
@@ -4158,8 +4164,8 @@
         <v>48.2</v>
       </c>
       <c r="S3" s="7">
-        <f>ATAN(TAN(R3*3.1415/180)-(1-Q3)/(2*(1+Q3)*P3))*180/3.1415</f>
-        <v>44.036243565531883</v>
+        <f t="shared" ref="S3:S11" si="7">ATAN(TAN(R3*3.1415/180)-(1-Q3)/((1+Q3)*P3))*180/3.1415</f>
+        <v>24.310202077346343</v>
       </c>
       <c r="T3" s="7">
         <v>1.1000000000000001</v>
@@ -4168,7 +4174,7 @@
         <v>25</v>
       </c>
       <c r="V3" s="7">
-        <f>U3*2</f>
+        <f t="shared" si="3"/>
         <v>50</v>
       </c>
       <c r="W3" s="7">
@@ -4181,7 +4187,7 @@
         <v>32</v>
       </c>
       <c r="Z3" s="7">
-        <f>(2/3)*((2*U3)/((SQRT(W3*U3))*(1+X3)))*(1+X3+X3^2)/(1+X3)</f>
+        <f t="shared" si="4"/>
         <v>3.171014677825942</v>
       </c>
       <c r="AA3" s="7">
@@ -4212,7 +4218,7 @@
         <v>55</v>
       </c>
       <c r="AJ3" s="7">
-        <f>2*AI3</f>
+        <f t="shared" si="5"/>
         <v>110</v>
       </c>
       <c r="AK3" s="7">
@@ -4225,7 +4231,7 @@
         <v>20</v>
       </c>
       <c r="AN3" s="7">
-        <f>(2/3)*((2*AI3)/((SQRT(AK3*AI3))*(1+AL3)))*(1+AL3+AL3^2)/(1+AL3)</f>
+        <f t="shared" si="6"/>
         <v>6.9026671531786787</v>
       </c>
       <c r="AO3" s="7">
@@ -4276,11 +4282,11 @@
         <v>5.5</v>
       </c>
       <c r="H4" s="7">
-        <f>F4/G4</f>
+        <f t="shared" si="0"/>
         <v>7.2727272727272725</v>
       </c>
       <c r="I4" s="7">
-        <f>((G4/2)^2)*3.1415+2.5</f>
+        <f t="shared" si="1"/>
         <v>26.257593750000002</v>
       </c>
       <c r="J4" s="7">
@@ -4297,14 +4303,14 @@
         <v>1</v>
       </c>
       <c r="N4" s="7">
-        <v>360</v>
+        <v>400</v>
       </c>
       <c r="O4" s="7">
-        <f>N4*2</f>
-        <v>720</v>
+        <f t="shared" si="2"/>
+        <v>800</v>
       </c>
       <c r="P4" s="7">
-        <v>2.2000000000000002</v>
+        <v>1</v>
       </c>
       <c r="Q4" s="7">
         <v>0.2</v>
@@ -4313,8 +4319,8 @@
         <v>48.2</v>
       </c>
       <c r="S4" s="7">
-        <f>ATAN(TAN(R4*3.1415/180)-(1-Q4)/(2*(1+Q4)*P4))*180/3.1415</f>
-        <v>44.036243565531883</v>
+        <f t="shared" si="7"/>
+        <v>24.310202077346343</v>
       </c>
       <c r="T4" s="7">
         <v>1.1000000000000001</v>
@@ -4323,7 +4329,7 @@
         <v>25</v>
       </c>
       <c r="V4" s="7">
-        <f>U4*2</f>
+        <f t="shared" si="3"/>
         <v>50</v>
       </c>
       <c r="W4" s="7">
@@ -4336,7 +4342,7 @@
         <v>32</v>
       </c>
       <c r="Z4" s="7">
-        <f>(2/3)*((2*U4)/((SQRT(W4*U4))*(1+X4)))*(1+X4+X4^2)/(1+X4)</f>
+        <f t="shared" si="4"/>
         <v>3.171014677825942</v>
       </c>
       <c r="AA4" s="7">
@@ -4367,7 +4373,7 @@
         <v>55</v>
       </c>
       <c r="AJ4" s="7">
-        <f>2*AI4</f>
+        <f t="shared" si="5"/>
         <v>110</v>
       </c>
       <c r="AK4" s="7">
@@ -4380,7 +4386,7 @@
         <v>20</v>
       </c>
       <c r="AN4" s="7">
-        <f>(2/3)*((2*AI4)/((SQRT(AK4*AI4))*(1+AL4)))*(1+AL4+AL4^2)/(1+AL4)</f>
+        <f t="shared" si="6"/>
         <v>6.9026671531786787</v>
       </c>
       <c r="AO4" s="7">
@@ -4431,11 +4437,11 @@
         <v>5.5</v>
       </c>
       <c r="H5" s="7">
-        <f>F5/G5</f>
+        <f t="shared" si="0"/>
         <v>7.2727272727272725</v>
       </c>
       <c r="I5" s="7">
-        <f>((G5/2)^2)*3.1415+2.5</f>
+        <f t="shared" si="1"/>
         <v>26.257593750000002</v>
       </c>
       <c r="J5" s="7">
@@ -4452,14 +4458,14 @@
         <v>1</v>
       </c>
       <c r="N5" s="7">
-        <v>360</v>
+        <v>350</v>
       </c>
       <c r="O5" s="7">
-        <f>N5*2</f>
-        <v>720</v>
+        <f t="shared" si="2"/>
+        <v>700</v>
       </c>
       <c r="P5" s="7">
-        <v>2.2000000000000002</v>
+        <v>1</v>
       </c>
       <c r="Q5" s="7">
         <v>0.2</v>
@@ -4468,8 +4474,8 @@
         <v>48.2</v>
       </c>
       <c r="S5" s="7">
-        <f>ATAN(TAN(R5*3.1415/180)-(1-Q5)/(2*(1+Q5)*P5))*180/3.1415</f>
-        <v>44.036243565531883</v>
+        <f t="shared" si="7"/>
+        <v>24.310202077346343</v>
       </c>
       <c r="T5" s="7">
         <v>1.1000000000000001</v>
@@ -4478,7 +4484,7 @@
         <v>25</v>
       </c>
       <c r="V5" s="7">
-        <f>U5*2</f>
+        <f t="shared" si="3"/>
         <v>50</v>
       </c>
       <c r="W5" s="7">
@@ -4491,7 +4497,7 @@
         <v>32</v>
       </c>
       <c r="Z5" s="7">
-        <f>(2/3)*((2*U5)/((SQRT(W5*U5))*(1+X5)))*(1+X5+X5^2)/(1+X5)</f>
+        <f t="shared" si="4"/>
         <v>3.171014677825942</v>
       </c>
       <c r="AA5" s="7">
@@ -4522,7 +4528,7 @@
         <v>55</v>
       </c>
       <c r="AJ5" s="7">
-        <f>2*AI5</f>
+        <f t="shared" si="5"/>
         <v>110</v>
       </c>
       <c r="AK5" s="7">
@@ -4535,7 +4541,7 @@
         <v>20</v>
       </c>
       <c r="AN5" s="7">
-        <f>(2/3)*((2*AI5)/((SQRT(AK5*AI5))*(1+AL5)))*(1+AL5+AL5^2)/(1+AL5)</f>
+        <f t="shared" si="6"/>
         <v>6.9026671531786787</v>
       </c>
       <c r="AO5" s="7">
@@ -4586,11 +4592,11 @@
         <v>5.5</v>
       </c>
       <c r="H6" s="7">
-        <f>F6/G6</f>
+        <f t="shared" si="0"/>
         <v>7.2727272727272725</v>
       </c>
       <c r="I6" s="7">
-        <f>((G6/2)^2)*3.1415+2.5</f>
+        <f t="shared" si="1"/>
         <v>26.257593750000002</v>
       </c>
       <c r="J6" s="7">
@@ -4607,14 +4613,14 @@
         <v>1</v>
       </c>
       <c r="N6" s="7">
-        <v>360</v>
+        <v>300</v>
       </c>
       <c r="O6" s="7">
-        <f>N6*2</f>
-        <v>720</v>
+        <f t="shared" si="2"/>
+        <v>600</v>
       </c>
       <c r="P6" s="7">
-        <v>2.2000000000000002</v>
+        <v>1</v>
       </c>
       <c r="Q6" s="7">
         <v>0.2</v>
@@ -4623,8 +4629,8 @@
         <v>48.2</v>
       </c>
       <c r="S6" s="7">
-        <f>ATAN(TAN(R6*3.1415/180)-(1-Q6)/(2*(1+Q6)*P6))*180/3.1415</f>
-        <v>44.036243565531883</v>
+        <f t="shared" si="7"/>
+        <v>24.310202077346343</v>
       </c>
       <c r="T6" s="7">
         <v>1.1000000000000001</v>
@@ -4633,7 +4639,7 @@
         <v>25</v>
       </c>
       <c r="V6" s="7">
-        <f>U6*2</f>
+        <f t="shared" si="3"/>
         <v>50</v>
       </c>
       <c r="W6" s="7">
@@ -4646,7 +4652,7 @@
         <v>32</v>
       </c>
       <c r="Z6" s="7">
-        <f>(2/3)*((2*U6)/((SQRT(W6*U6))*(1+X6)))*(1+X6+X6^2)/(1+X6)</f>
+        <f t="shared" si="4"/>
         <v>3.171014677825942</v>
       </c>
       <c r="AA6" s="7">
@@ -4677,7 +4683,7 @@
         <v>55</v>
       </c>
       <c r="AJ6" s="7">
-        <f>2*AI6</f>
+        <f t="shared" si="5"/>
         <v>110</v>
       </c>
       <c r="AK6" s="7">
@@ -4690,7 +4696,7 @@
         <v>20</v>
       </c>
       <c r="AN6" s="7">
-        <f>(2/3)*((2*AI6)/((SQRT(AK6*AI6))*(1+AL6)))*(1+AL6+AL6^2)/(1+AL6)</f>
+        <f t="shared" si="6"/>
         <v>6.9026671531786787</v>
       </c>
       <c r="AO6" s="7">
@@ -4741,11 +4747,11 @@
         <v>4.5</v>
       </c>
       <c r="H7" s="7">
-        <f>F7/G7</f>
+        <f t="shared" si="0"/>
         <v>5.5555555555555554</v>
       </c>
       <c r="I7" s="7">
-        <f>((G7/2)^2)*3.1415+2.5</f>
+        <f t="shared" si="1"/>
         <v>18.40384375</v>
       </c>
       <c r="J7" s="7">
@@ -4765,7 +4771,7 @@
         <v>310</v>
       </c>
       <c r="O7" s="7">
-        <f>N7*2</f>
+        <f t="shared" si="2"/>
         <v>620</v>
       </c>
       <c r="P7" s="7">
@@ -4778,8 +4784,8 @@
         <v>44</v>
       </c>
       <c r="S7" s="7">
-        <f>ATAN(TAN(R7*3.1415/180)-(1-Q7)/(2*(1+Q7)*P7))*180/3.1415</f>
-        <v>40.208174924683249</v>
+        <f t="shared" si="7"/>
+        <v>35.939576280851796</v>
       </c>
       <c r="T7" s="7">
         <v>1.1000000000000001</v>
@@ -4788,7 +4794,7 @@
         <v>10</v>
       </c>
       <c r="V7" s="7">
-        <f>U7*2</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="W7" s="7">
@@ -4801,7 +4807,7 @@
         <v>31</v>
       </c>
       <c r="Z7" s="7">
-        <f>(2/3)*((2*U7)/((SQRT(W7*U7))*(1+X7)))*(1+X7+X7^2)/(1+X7)</f>
+        <f t="shared" si="4"/>
         <v>1.6237266827246648</v>
       </c>
       <c r="AA7" s="7">
@@ -4832,7 +4838,7 @@
         <v>17</v>
       </c>
       <c r="AJ7" s="7">
-        <f>2*AI7</f>
+        <f t="shared" si="5"/>
         <v>34</v>
       </c>
       <c r="AK7" s="7">
@@ -4845,7 +4851,7 @@
         <v>20</v>
       </c>
       <c r="AN7" s="7">
-        <f>(2/3)*((2*AI7)/((SQRT(AK7*AI7))*(1+AL7)))*(1+AL7+AL7^2)/(1+AL7)</f>
+        <f t="shared" si="6"/>
         <v>3.2613354542804762</v>
       </c>
       <c r="AO7" s="7">
@@ -4896,11 +4902,11 @@
         <v>4.5</v>
       </c>
       <c r="H8" s="7">
-        <f>F8/G8</f>
+        <f t="shared" si="0"/>
         <v>5.5555555555555554</v>
       </c>
       <c r="I8" s="7">
-        <f>((G8/2)^2)*3.1415+2.5</f>
+        <f t="shared" si="1"/>
         <v>18.40384375</v>
       </c>
       <c r="J8" s="7">
@@ -4920,7 +4926,7 @@
         <v>310</v>
       </c>
       <c r="O8" s="7">
-        <f>N8*2</f>
+        <f t="shared" si="2"/>
         <v>620</v>
       </c>
       <c r="P8" s="7">
@@ -4933,8 +4939,8 @@
         <v>44</v>
       </c>
       <c r="S8" s="7">
-        <f>ATAN(TAN(R8*3.1415/180)-(1-Q8)/(2*(1+Q8)*P8))*180/3.1415</f>
-        <v>40.208174924683249</v>
+        <f t="shared" si="7"/>
+        <v>35.939576280851796</v>
       </c>
       <c r="T8" s="7">
         <v>1.1000000000000001</v>
@@ -4943,7 +4949,7 @@
         <v>10</v>
       </c>
       <c r="V8" s="7">
-        <f>U8*2</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="W8" s="7">
@@ -4956,7 +4962,7 @@
         <v>31</v>
       </c>
       <c r="Z8" s="7">
-        <f>(2/3)*((2*U8)/((SQRT(W8*U8))*(1+X8)))*(1+X8+X8^2)/(1+X8)</f>
+        <f t="shared" si="4"/>
         <v>1.6237266827246648</v>
       </c>
       <c r="AA8" s="7">
@@ -4987,7 +4993,7 @@
         <v>17</v>
       </c>
       <c r="AJ8" s="7">
-        <f>2*AI8</f>
+        <f t="shared" si="5"/>
         <v>34</v>
       </c>
       <c r="AK8" s="7">
@@ -5000,7 +5006,7 @@
         <v>20</v>
       </c>
       <c r="AN8" s="7">
-        <f>(2/3)*((2*AI8)/((SQRT(AK8*AI8))*(1+AL8)))*(1+AL8+AL8^2)/(1+AL8)</f>
+        <f t="shared" si="6"/>
         <v>3.2613354542804762</v>
       </c>
       <c r="AO8" s="7">
@@ -5051,11 +5057,11 @@
         <v>4.5</v>
       </c>
       <c r="H9" s="7">
-        <f>F9/G9</f>
+        <f t="shared" si="0"/>
         <v>5.5555555555555554</v>
       </c>
       <c r="I9" s="7">
-        <f>((G9/2)^2)*3.1415+2.5</f>
+        <f t="shared" si="1"/>
         <v>18.40384375</v>
       </c>
       <c r="J9" s="7">
@@ -5075,7 +5081,7 @@
         <v>310</v>
       </c>
       <c r="O9" s="7">
-        <f>N9*2</f>
+        <f t="shared" si="2"/>
         <v>620</v>
       </c>
       <c r="P9" s="7">
@@ -5088,8 +5094,8 @@
         <v>44</v>
       </c>
       <c r="S9" s="7">
-        <f>ATAN(TAN(R9*3.1415/180)-(1-Q9)/(2*(1+Q9)*P9))*180/3.1415</f>
-        <v>40.208174924683249</v>
+        <f t="shared" si="7"/>
+        <v>35.939576280851796</v>
       </c>
       <c r="T9" s="7">
         <v>1.1000000000000001</v>
@@ -5098,7 +5104,7 @@
         <v>10</v>
       </c>
       <c r="V9" s="7">
-        <f>U9*2</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="W9" s="7">
@@ -5111,7 +5117,7 @@
         <v>31</v>
       </c>
       <c r="Z9" s="7">
-        <f>(2/3)*((2*U9)/((SQRT(W9*U9))*(1+X9)))*(1+X9+X9^2)/(1+X9)</f>
+        <f t="shared" si="4"/>
         <v>1.6237266827246648</v>
       </c>
       <c r="AA9" s="7">
@@ -5142,7 +5148,7 @@
         <v>17</v>
       </c>
       <c r="AJ9" s="7">
-        <f>2*AI9</f>
+        <f t="shared" si="5"/>
         <v>34</v>
       </c>
       <c r="AK9" s="7">
@@ -5155,7 +5161,7 @@
         <v>20</v>
       </c>
       <c r="AN9" s="7">
-        <f>(2/3)*((2*AI9)/((SQRT(AK9*AI9))*(1+AL9)))*(1+AL9+AL9^2)/(1+AL9)</f>
+        <f t="shared" si="6"/>
         <v>3.2613354542804762</v>
       </c>
       <c r="AO9" s="7">
@@ -5206,11 +5212,11 @@
         <v>4.5</v>
       </c>
       <c r="H10" s="7">
-        <f>F10/G10</f>
+        <f t="shared" si="0"/>
         <v>5.5555555555555554</v>
       </c>
       <c r="I10" s="7">
-        <f>((G10/2)^2)*3.1415+2.5</f>
+        <f t="shared" si="1"/>
         <v>18.40384375</v>
       </c>
       <c r="J10" s="7">
@@ -5230,7 +5236,7 @@
         <v>310</v>
       </c>
       <c r="O10" s="7">
-        <f>N10*2</f>
+        <f t="shared" si="2"/>
         <v>620</v>
       </c>
       <c r="P10" s="7">
@@ -5243,8 +5249,8 @@
         <v>44</v>
       </c>
       <c r="S10" s="7">
-        <f>ATAN(TAN(R10*3.1415/180)-(1-Q10)/(2*(1+Q10)*P10))*180/3.1415</f>
-        <v>40.208174924683249</v>
+        <f t="shared" si="7"/>
+        <v>35.939576280851796</v>
       </c>
       <c r="T10" s="7">
         <v>1.1000000000000001</v>
@@ -5253,7 +5259,7 @@
         <v>10</v>
       </c>
       <c r="V10" s="7">
-        <f>U10*2</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="W10" s="7">
@@ -5266,7 +5272,7 @@
         <v>31</v>
       </c>
       <c r="Z10" s="7">
-        <f>(2/3)*((2*U10)/((SQRT(W10*U10))*(1+X10)))*(1+X10+X10^2)/(1+X10)</f>
+        <f t="shared" si="4"/>
         <v>1.6237266827246648</v>
       </c>
       <c r="AA10" s="7">
@@ -5297,7 +5303,7 @@
         <v>17</v>
       </c>
       <c r="AJ10" s="7">
-        <f>2*AI10</f>
+        <f t="shared" si="5"/>
         <v>34</v>
       </c>
       <c r="AK10" s="7">
@@ -5310,7 +5316,7 @@
         <v>20</v>
       </c>
       <c r="AN10" s="7">
-        <f>(2/3)*((2*AI10)/((SQRT(AK10*AI10))*(1+AL10)))*(1+AL10+AL10^2)/(1+AL10)</f>
+        <f t="shared" si="6"/>
         <v>3.2613354542804762</v>
       </c>
       <c r="AO10" s="7">
@@ -5361,11 +5367,11 @@
         <v>4.5</v>
       </c>
       <c r="H11" s="7">
-        <f>F11/G11</f>
+        <f t="shared" si="0"/>
         <v>5.5555555555555554</v>
       </c>
       <c r="I11" s="7">
-        <f>((G11/2)^2)*3.1415+2.5</f>
+        <f t="shared" si="1"/>
         <v>18.40384375</v>
       </c>
       <c r="J11" s="7">
@@ -5385,7 +5391,7 @@
         <v>310</v>
       </c>
       <c r="O11" s="7">
-        <f>N11*2</f>
+        <f t="shared" si="2"/>
         <v>620</v>
       </c>
       <c r="P11" s="7">
@@ -5398,8 +5404,8 @@
         <v>44</v>
       </c>
       <c r="S11" s="7">
-        <f>ATAN(TAN(R11*3.1415/180)-(1-Q11)/(2*(1+Q11)*P11))*180/3.1415</f>
-        <v>40.208174924683249</v>
+        <f t="shared" si="7"/>
+        <v>35.939576280851796</v>
       </c>
       <c r="T11" s="7">
         <v>1.1000000000000001</v>
@@ -5408,7 +5414,7 @@
         <v>10</v>
       </c>
       <c r="V11" s="7">
-        <f>U11*2</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="W11" s="7">
@@ -5421,7 +5427,7 @@
         <v>31</v>
       </c>
       <c r="Z11" s="7">
-        <f>(2/3)*((2*U11)/((SQRT(W11*U11))*(1+X11)))*(1+X11+X11^2)/(1+X11)</f>
+        <f t="shared" si="4"/>
         <v>1.6237266827246648</v>
       </c>
       <c r="AA11" s="7">
@@ -5452,7 +5458,7 @@
         <v>17</v>
       </c>
       <c r="AJ11" s="7">
-        <f>2*AI11</f>
+        <f t="shared" si="5"/>
         <v>34</v>
       </c>
       <c r="AK11" s="7">
@@ -5465,7 +5471,7 @@
         <v>20</v>
       </c>
       <c r="AN11" s="7">
-        <f>(2/3)*((2*AI11)/((SQRT(AK11*AI11))*(1+AL11)))*(1+AL11+AL11^2)/(1+AL11)</f>
+        <f t="shared" si="6"/>
         <v>3.2613354542804762</v>
       </c>
       <c r="AO11" s="7">
@@ -5494,6 +5500,476 @@
       </c>
     </row>
     <row r="15" spans="1:48" s="20" customFormat="1"/>
+    <row r="16" spans="1:48">
+      <c r="A16" s="7" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="17" spans="1:48">
+      <c r="A17" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C17" s="7">
+        <v>0</v>
+      </c>
+      <c r="D17" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="E17" s="7">
+        <v>1</v>
+      </c>
+      <c r="F17" s="7">
+        <v>45</v>
+      </c>
+      <c r="G17" s="7">
+        <v>5.5</v>
+      </c>
+      <c r="H17" s="7">
+        <f t="shared" ref="H17" si="8">F17/G17</f>
+        <v>8.1818181818181817</v>
+      </c>
+      <c r="I17" s="7">
+        <f t="shared" ref="I17" si="9">((G17/2)^2)*3.1415+2.5</f>
+        <v>26.257593750000002</v>
+      </c>
+      <c r="J17" s="7">
+        <v>0</v>
+      </c>
+      <c r="K17" s="7">
+        <f>(F17)*G17*3.1415*0.9</f>
+        <v>699.76912500000003</v>
+      </c>
+      <c r="L17" s="7">
+        <v>1</v>
+      </c>
+      <c r="M17" s="7">
+        <v>1</v>
+      </c>
+      <c r="N17" s="7">
+        <v>450</v>
+      </c>
+      <c r="O17" s="7">
+        <f t="shared" ref="O17" si="10">N17*2</f>
+        <v>900</v>
+      </c>
+      <c r="P17" s="7">
+        <v>3.63</v>
+      </c>
+      <c r="Q17" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="R17" s="7">
+        <v>34</v>
+      </c>
+      <c r="S17" s="7">
+        <f>ATAN(TAN(R17*3.1415/180)-(1-Q17)/((1+Q17)*P17))*180/3.1415</f>
+        <v>26.143883229632934</v>
+      </c>
+      <c r="T17" s="7">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="U17" s="7">
+        <v>25</v>
+      </c>
+      <c r="V17" s="7">
+        <f t="shared" ref="V17" si="11">U17*2</f>
+        <v>50</v>
+      </c>
+      <c r="W17" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="X17" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="Y17" s="7">
+        <v>32</v>
+      </c>
+      <c r="Z17" s="7">
+        <f t="shared" ref="Z17" si="12">(2/3)*((2*U17)/((SQRT(W17*U17))*(1+X17)))*(1+X17+X17^2)/(1+X17)</f>
+        <v>3.171014677825942</v>
+      </c>
+      <c r="AA17" s="7">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AB17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AC17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AD17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AE17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AG17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AH17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AI17" s="7">
+        <v>55</v>
+      </c>
+      <c r="AJ17" s="7">
+        <f t="shared" ref="AJ17" si="13">2*AI17</f>
+        <v>110</v>
+      </c>
+      <c r="AK17" s="7">
+        <v>1.3</v>
+      </c>
+      <c r="AL17" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AM17" s="7">
+        <v>20</v>
+      </c>
+      <c r="AN17" s="7">
+        <f t="shared" ref="AN17" si="14">(2/3)*((2*AI17)/((SQRT(AK17*AI17))*(1+AL17)))*(1+AL17+AL17^2)/(1+AL17)</f>
+        <v>6.9026671531786787</v>
+      </c>
+      <c r="AO17" s="7">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AP17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AQ17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AR17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AS17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AT17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AU17" s="7">
+        <v>0</v>
+      </c>
+      <c r="AV17" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:48">
+      <c r="A18" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C18" s="7">
+        <v>0</v>
+      </c>
+      <c r="D18" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="E18" s="7">
+        <v>1</v>
+      </c>
+      <c r="F18" s="7">
+        <v>40</v>
+      </c>
+      <c r="G18" s="7">
+        <v>5.5</v>
+      </c>
+      <c r="H18" s="7">
+        <f t="shared" ref="H18:H19" si="15">F18/G18</f>
+        <v>7.2727272727272725</v>
+      </c>
+      <c r="I18" s="7">
+        <f t="shared" ref="I18:I19" si="16">((G18/2)^2)*3.1415+2.5</f>
+        <v>26.257593750000002</v>
+      </c>
+      <c r="J18" s="7">
+        <v>0</v>
+      </c>
+      <c r="K18" s="7">
+        <f>(F18)*G18*3.1415*0.9</f>
+        <v>622.01700000000005</v>
+      </c>
+      <c r="L18" s="7">
+        <v>1</v>
+      </c>
+      <c r="M18" s="7">
+        <v>1</v>
+      </c>
+      <c r="N18" s="7">
+        <v>380</v>
+      </c>
+      <c r="O18" s="7">
+        <f t="shared" ref="O18:O19" si="17">N18*2</f>
+        <v>760</v>
+      </c>
+      <c r="P18" s="7">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="Q18" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="R18" s="7">
+        <v>34</v>
+      </c>
+      <c r="S18" s="7">
+        <f t="shared" ref="S18:S19" si="18">ATAN(TAN(R18*3.1415/180)-(1-Q18)/((1+Q18)*P18))*180/3.1415</f>
+        <v>20.378253616689143</v>
+      </c>
+      <c r="T18" s="7">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="U18" s="7">
+        <v>25</v>
+      </c>
+      <c r="V18" s="7">
+        <f t="shared" ref="V18:V19" si="19">U18*2</f>
+        <v>50</v>
+      </c>
+      <c r="W18" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="X18" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="Y18" s="7">
+        <v>32</v>
+      </c>
+      <c r="Z18" s="7">
+        <f t="shared" ref="Z18:Z19" si="20">(2/3)*((2*U18)/((SQRT(W18*U18))*(1+X18)))*(1+X18+X18^2)/(1+X18)</f>
+        <v>3.171014677825942</v>
+      </c>
+      <c r="AA18" s="7">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AB18" s="7">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="7">
+        <v>0</v>
+      </c>
+      <c r="AD18" s="7">
+        <v>0</v>
+      </c>
+      <c r="AE18" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF18" s="7">
+        <v>0</v>
+      </c>
+      <c r="AG18" s="7">
+        <v>0</v>
+      </c>
+      <c r="AH18" s="7">
+        <v>0</v>
+      </c>
+      <c r="AI18" s="7">
+        <v>55</v>
+      </c>
+      <c r="AJ18" s="7">
+        <f t="shared" ref="AJ18:AJ19" si="21">2*AI18</f>
+        <v>110</v>
+      </c>
+      <c r="AK18" s="7">
+        <v>1.3</v>
+      </c>
+      <c r="AL18" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AM18" s="7">
+        <v>20</v>
+      </c>
+      <c r="AN18" s="7">
+        <f t="shared" ref="AN18:AN19" si="22">(2/3)*((2*AI18)/((SQRT(AK18*AI18))*(1+AL18)))*(1+AL18+AL18^2)/(1+AL18)</f>
+        <v>6.9026671531786787</v>
+      </c>
+      <c r="AO18" s="7">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AP18" s="7">
+        <v>0</v>
+      </c>
+      <c r="AQ18" s="7">
+        <v>0</v>
+      </c>
+      <c r="AR18" s="7">
+        <v>0</v>
+      </c>
+      <c r="AS18" s="7">
+        <v>0</v>
+      </c>
+      <c r="AT18" s="7">
+        <v>0</v>
+      </c>
+      <c r="AU18" s="7">
+        <v>0</v>
+      </c>
+      <c r="AV18" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:48">
+      <c r="A19" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C19" s="7">
+        <v>0</v>
+      </c>
+      <c r="D19" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="E19" s="7">
+        <v>1</v>
+      </c>
+      <c r="F19" s="7">
+        <v>40</v>
+      </c>
+      <c r="G19" s="7">
+        <v>5.5</v>
+      </c>
+      <c r="H19" s="7">
+        <f t="shared" si="15"/>
+        <v>7.2727272727272725</v>
+      </c>
+      <c r="I19" s="7">
+        <f t="shared" si="16"/>
+        <v>26.257593750000002</v>
+      </c>
+      <c r="J19" s="7">
+        <v>0</v>
+      </c>
+      <c r="K19" s="7">
+        <f>(F19)*G19*3.1415*0.9</f>
+        <v>622.01700000000005</v>
+      </c>
+      <c r="L19" s="7">
+        <v>1</v>
+      </c>
+      <c r="M19" s="7">
+        <v>1</v>
+      </c>
+      <c r="N19" s="7">
+        <v>360</v>
+      </c>
+      <c r="O19" s="7">
+        <f t="shared" si="17"/>
+        <v>720</v>
+      </c>
+      <c r="P19" s="7">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="Q19" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="R19" s="7">
+        <v>48.2</v>
+      </c>
+      <c r="S19" s="7">
+        <f t="shared" si="18"/>
+        <v>39.193340519780634</v>
+      </c>
+      <c r="T19" s="7">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="U19" s="7">
+        <v>25</v>
+      </c>
+      <c r="V19" s="7">
+        <f t="shared" si="19"/>
+        <v>50</v>
+      </c>
+      <c r="W19" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="X19" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="Y19" s="7">
+        <v>32</v>
+      </c>
+      <c r="Z19" s="7">
+        <f t="shared" si="20"/>
+        <v>3.171014677825942</v>
+      </c>
+      <c r="AA19" s="7">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AB19" s="7">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="7">
+        <v>0</v>
+      </c>
+      <c r="AD19" s="7">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF19" s="7">
+        <v>0</v>
+      </c>
+      <c r="AG19" s="7">
+        <v>0</v>
+      </c>
+      <c r="AH19" s="7">
+        <v>0</v>
+      </c>
+      <c r="AI19" s="7">
+        <v>55</v>
+      </c>
+      <c r="AJ19" s="7">
+        <f t="shared" si="21"/>
+        <v>110</v>
+      </c>
+      <c r="AK19" s="7">
+        <v>1.3</v>
+      </c>
+      <c r="AL19" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AM19" s="7">
+        <v>20</v>
+      </c>
+      <c r="AN19" s="7">
+        <f t="shared" si="22"/>
+        <v>6.9026671531786787</v>
+      </c>
+      <c r="AO19" s="7">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="AP19" s="7">
+        <v>0</v>
+      </c>
+      <c r="AQ19" s="7">
+        <v>0</v>
+      </c>
+      <c r="AR19" s="7">
+        <v>0</v>
+      </c>
+      <c r="AS19" s="7">
+        <v>0</v>
+      </c>
+      <c r="AT19" s="7">
+        <v>0</v>
+      </c>
+      <c r="AU19" s="7">
+        <v>0</v>
+      </c>
+      <c r="AV19" s="7">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -5507,7 +5983,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>B2:B14</xm:sqref>
+          <xm:sqref>B2:B14 B17:B19</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -7523,7 +7999,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:R18"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
@@ -8179,6 +8655,125 @@
       <c r="A14" s="21"/>
     </row>
     <row r="15" spans="1:18" s="12" customFormat="1"/>
+    <row r="16" spans="1:18">
+      <c r="A16" s="7" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18">
+      <c r="A17" t="s">
+        <v>249</v>
+      </c>
+      <c r="B17" t="s">
+        <v>214</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
+      </c>
+      <c r="D17">
+        <v>6500</v>
+      </c>
+      <c r="E17">
+        <v>0.77</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0.2</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <f>M17*N17*O17*P17</f>
+        <v>0</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18">
+      <c r="A18" t="s">
+        <v>242</v>
+      </c>
+      <c r="B18" t="s">
+        <v>214</v>
+      </c>
+      <c r="C18">
+        <v>2</v>
+      </c>
+      <c r="D18">
+        <v>5500</v>
+      </c>
+      <c r="E18">
+        <v>0.77</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0.2</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <v>0</v>
+      </c>
+      <c r="Q18">
+        <f>M18*N18*O18*P18</f>
+        <v>0</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>